<commit_message>
feat: add subtitle, responsibilities, and programs fields to divisions; update related queries and requests
</commit_message>
<xml_diff>
--- a/docs/templates/template_import_divisions.xlsx
+++ b/docs/templates/template_import_divisions.xlsx
@@ -72,7 +72,7 @@
             <b val="1"/>
             <color/>
           </rPr>
-          <t xml:space="preserve">description
+          <t xml:space="preserve">subtitle
 </t>
         </r>
         <r>
@@ -82,7 +82,7 @@
             <color indexed="81"/>
             <sz val="9"/>
           </rPr>
-          <t xml:space="preserve">Penjelasan tugas dan cakupan kerja divisi.</t>
+          <t xml:space="preserve">Kalimat singkat yang tampil pada hero halaman detail divisi.</t>
         </r>
       </text>
     </comment>
@@ -94,7 +94,7 @@
             <b val="1"/>
             <color/>
           </rPr>
-          <t xml:space="preserve">coordinator_nim
+          <t xml:space="preserve">description
 </t>
         </r>
         <r>
@@ -104,11 +104,77 @@
             <color indexed="81"/>
             <sz val="9"/>
           </rPr>
-          <t xml:space="preserve">NIM anggota yang menjadi koordinator. Anggota harus sudah terdaftar. Kosongkan bila belum ditentukan.</t>
+          <t xml:space="preserve">Penjelasan tugas dan cakupan kerja divisi.</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <family val="2"/>
+            <b val="1"/>
+            <color/>
+          </rPr>
+          <t xml:space="preserve">responsibilities
+</t>
+        </r>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <color indexed="81"/>
+            <sz val="9"/>
+          </rPr>
+          <t xml:space="preserve">Daftar tanggung jawab divisi. Pisahkan antar butir dengan tanda titik koma (;).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <family val="2"/>
+            <b val="1"/>
+            <color/>
+          </rPr>
+          <t xml:space="preserve">programs
+</t>
+        </r>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <color indexed="81"/>
+            <sz val="9"/>
+          </rPr>
+          <t xml:space="preserve">Daftar program kerja. Tulis tiap program dengan format Nama | Deskripsi, lalu pisahkan antar program dengan tanda titik koma (;).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <family val="2"/>
+            <b val="1"/>
+            <color/>
+          </rPr>
+          <t xml:space="preserve">coordinator_nim
+</t>
+        </r>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <color indexed="81"/>
+            <sz val="9"/>
+          </rPr>
+          <t xml:space="preserve">NIM anggota yang menjadi koordinator. Anggota harus sudah terdaftar. Kosongkan bila belum ditentukan.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -135,7 +201,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>name</t>
   </si>
@@ -155,13 +221,31 @@
     <t>humas</t>
   </si>
   <si>
+    <t>subtitle</t>
+  </si>
+  <si>
+    <t>Wajah KMH di dunia digital.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>description</t>
   </si>
   <si>
     <t>Mengelola konten dan publikasi KMH.</t>
   </si>
   <si>
-    <t/>
+    <t>responsibilities</t>
+  </si>
+  <si>
+    <t>Mengelola media sosial KMH; Membuat konten publikasi kegiatan</t>
+  </si>
+  <si>
+    <t>programs</t>
+  </si>
+  <si>
+    <t>KMH Podcast | Podcast bulanan seputar kegiatan KMH; Kelas Desain | Pelatihan desain untuk anggota</t>
   </si>
   <si>
     <t>coordinator_nim</t>
@@ -239,7 +323,16 @@
     <t>opsional</t>
   </si>
   <si>
+    <t>Kalimat singkat yang tampil pada hero halaman detail divisi.</t>
+  </si>
+  <si>
     <t>Penjelasan tugas dan cakupan kerja divisi.</t>
+  </si>
+  <si>
+    <t>Daftar tanggung jawab divisi. Pisahkan antar butir dengan tanda titik koma (;).</t>
+  </si>
+  <si>
+    <t>Daftar program kerja. Tulis tiap program dengan format Nama | Deskripsi, lalu pisahkan antar program dengan tanda titik koma (;).</t>
   </si>
   <si>
     <t>NIM anggota yang menjadi koordinator. Anggota harus sudah terdaftar. Kosongkan bila belum ditentukan.</t>
@@ -588,10 +681,12 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="2" min="1" width="16"/>
-    <col customWidth="true" max="3" min="3" width="17"/>
-    <col customWidth="true" max="4" min="4" width="21"/>
-    <col customWidth="true" max="5" min="5" width="16"/>
+    <col customWidth="true" max="3" min="1" width="16"/>
+    <col customWidth="true" max="4" min="4" width="17"/>
+    <col customWidth="true" max="5" min="5" width="22"/>
+    <col customWidth="true" max="6" min="6" width="16"/>
+    <col customWidth="true" max="7" min="7" width="21"/>
+    <col customWidth="true" max="8" min="8" width="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -610,6 +705,15 @@
       <c r="E1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -627,6 +731,15 @@
       <c r="E2" t="s">
         <v>12</v>
       </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -642,7 +755,16 @@
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -662,76 +784,76 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16">
@@ -739,13 +861,13 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17">
@@ -753,13 +875,13 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18">
@@ -767,13 +889,13 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -781,13 +903,13 @@
         <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20">
@@ -795,13 +917,55 @@
         <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
         <v>36</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>37</v>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add division_type field to divisions and update related queries and services
</commit_message>
<xml_diff>
--- a/docs/templates/template_import_divisions.xlsx
+++ b/docs/templates/template_import_divisions.xlsx
@@ -116,7 +116,7 @@
             <b val="1"/>
             <color/>
           </rPr>
-          <t xml:space="preserve">responsibilities
+          <t xml:space="preserve">division_type
 </t>
         </r>
         <r>
@@ -126,7 +126,7 @@
             <color indexed="81"/>
             <sz val="9"/>
           </rPr>
-          <t xml:space="preserve">Daftar tanggung jawab divisi. Pisahkan antar butir dengan tanda titik koma (;).</t>
+          <t xml:space="preserve">Tipe divisi: internal (di bawah Wakil Ketua Internal) atau external (di bawah Wakil Ketua External). Kosong dianggap internal.</t>
         </r>
       </text>
     </comment>
@@ -138,7 +138,7 @@
             <b val="1"/>
             <color/>
           </rPr>
-          <t xml:space="preserve">programs
+          <t xml:space="preserve">responsibilities
 </t>
         </r>
         <r>
@@ -148,7 +148,7 @@
             <color indexed="81"/>
             <sz val="9"/>
           </rPr>
-          <t xml:space="preserve">Daftar program kerja. Tulis tiap program dengan format Nama | Deskripsi, lalu pisahkan antar program dengan tanda titik koma (;).</t>
+          <t xml:space="preserve">Daftar tanggung jawab divisi. Pisahkan antar butir dengan tanda titik koma (;).</t>
         </r>
       </text>
     </comment>
@@ -160,7 +160,7 @@
             <b val="1"/>
             <color/>
           </rPr>
-          <t xml:space="preserve">coordinator_nim
+          <t xml:space="preserve">programs
 </t>
         </r>
         <r>
@@ -170,11 +170,33 @@
             <color indexed="81"/>
             <sz val="9"/>
           </rPr>
-          <t xml:space="preserve">NIM anggota yang menjadi koordinator. Anggota harus sudah terdaftar. Kosongkan bila belum ditentukan.</t>
+          <t xml:space="preserve">Daftar program kerja. Tulis tiap program dengan format Nama | Deskripsi, lalu pisahkan antar program dengan tanda titik koma (;).</t>
         </r>
       </text>
     </comment>
     <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <family val="2"/>
+            <b val="1"/>
+            <color/>
+          </rPr>
+          <t xml:space="preserve">coordinator_nim
+</t>
+        </r>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <color indexed="81"/>
+            <sz val="9"/>
+          </rPr>
+          <t xml:space="preserve">NIM anggota yang menjadi koordinator. Anggota harus sudah terdaftar. Kosongkan bila belum ditentukan.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -201,7 +223,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>name</t>
   </si>
@@ -236,6 +258,15 @@
     <t>Mengelola konten dan publikasi KMH.</t>
   </si>
   <si>
+    <t>division_type</t>
+  </si>
+  <si>
+    <t>internal</t>
+  </si>
+  <si>
+    <t>external</t>
+  </si>
+  <si>
     <t>responsibilities</t>
   </si>
   <si>
@@ -327,6 +358,9 @@
   </si>
   <si>
     <t>Penjelasan tugas dan cakupan kerja divisi.</t>
+  </si>
+  <si>
+    <t>Tipe divisi: internal (di bawah Wakil Ketua Internal) atau external (di bawah Wakil Ketua External). Kosong dianggap internal.</t>
   </si>
   <si>
     <t>Daftar tanggung jawab divisi. Pisahkan antar butir dengan tanda titik koma (;).</t>
@@ -683,10 +717,11 @@
   <cols>
     <col customWidth="true" max="3" min="1" width="16"/>
     <col customWidth="true" max="4" min="4" width="17"/>
-    <col customWidth="true" max="5" min="5" width="22"/>
-    <col customWidth="true" max="6" min="6" width="16"/>
-    <col customWidth="true" max="7" min="7" width="21"/>
-    <col customWidth="true" max="8" min="8" width="16"/>
+    <col customWidth="true" max="5" min="5" width="19"/>
+    <col customWidth="true" max="6" min="6" width="22"/>
+    <col customWidth="true" max="7" min="7" width="16"/>
+    <col customWidth="true" max="8" min="8" width="21"/>
+    <col customWidth="true" max="9" min="9" width="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -706,13 +741,16 @@
         <v>11</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="2">
@@ -732,13 +770,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -755,7 +796,7 @@
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
@@ -764,7 +805,10 @@
         <v>8</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>8</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -784,76 +828,76 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16">
@@ -861,13 +905,13 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -875,13 +919,13 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18">
@@ -889,13 +933,13 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" t="s">
         <v>39</v>
       </c>
-      <c r="C18" t="s">
-        <v>36</v>
-      </c>
       <c r="D18" s="3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19">
@@ -903,13 +947,13 @@
         <v>9</v>
       </c>
       <c r="B19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" t="s">
         <v>39</v>
       </c>
-      <c r="C19" t="s">
-        <v>36</v>
-      </c>
       <c r="D19" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20">
@@ -917,55 +961,69 @@
         <v>11</v>
       </c>
       <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" t="s">
         <v>39</v>
       </c>
-      <c r="C20" t="s">
-        <v>36</v>
-      </c>
       <c r="D20" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" t="s">
         <v>39</v>
       </c>
-      <c r="C21" t="s">
-        <v>36</v>
-      </c>
       <c r="D21" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" t="s">
         <v>39</v>
       </c>
-      <c r="C22" t="s">
-        <v>36</v>
-      </c>
       <c r="D22" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" t="s">
         <v>39</v>
       </c>
-      <c r="C23" t="s">
-        <v>45</v>
-      </c>
       <c r="D23" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>